<commit_message>
Update CORE-000249 rule and negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000249/negative/03/data/unit-test-CG0032-negative.xlsx
+++ b/rules/CORE-000249/negative/03/data/unit-test-CG0032-negative.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JanakiRaman\CORE\Rule_Authoring\core-contributor\rules\CORE-000249\negative\03\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A04D965D-B813-46A7-81DE-AF2424C73A23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10C1B25-30D6-43DD-A7E5-70CEAD7DEF44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="165">
   <si>
     <t>Product</t>
   </si>
@@ -516,6 +516,9 @@
   </si>
   <si>
     <t>Record</t>
+  </si>
+  <si>
+    <t>TV.VISITDY</t>
   </si>
 </sst>
 </file>
@@ -588,7 +591,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -604,6 +607,9 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -968,11 +974,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1006,13 +1012,13 @@
         <v>163</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2">
-        <v>99999</v>
+        <v>41</v>
+      </c>
+      <c r="F2" s="6">
+        <v>-15</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -1026,13 +1032,13 @@
         <v>163</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="6">
-        <v>-15</v>
+        <v>38</v>
+      </c>
+      <c r="F3">
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -1049,30 +1055,10 @@
         <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5">
+        <v>164</v>
+      </c>
+      <c r="F4" s="6">
         <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D5">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F5" s="6">
-        <v>-15</v>
       </c>
     </row>
   </sheetData>
@@ -1454,7 +1440,7 @@
       <c r="V5" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="W5" s="5" t="s">
+      <c r="W5" s="7" t="s">
         <v>82</v>
       </c>
       <c r="X5" s="4" t="s">
@@ -1463,7 +1449,7 @@
       <c r="Y5" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="Z5" s="5">
+      <c r="Z5" s="7">
         <v>-15</v>
       </c>
     </row>

</xml_diff>